<commit_message>
1.1.8 New field on label
</commit_message>
<xml_diff>
--- a/Data/InputData.xlsx
+++ b/Data/InputData.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27425"/>
-  <workbookPr defaultThemeVersion="202300"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
+  <workbookPr codeName="ThisWorkbook" defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\lenna\OneDrive\Documenten\Bureaublad\Archive\Werk\Marvu\Automatiseringen\Print Labels\Data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\lenna\Desktop\MS\Marvu\RPA\Print Labels\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2CC1F656-419D-49F3-B7BF-79C3E845B31A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A98E1AFA-2358-4B2C-B216-ED8997D03F4A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="780" yWindow="780" windowWidth="38700" windowHeight="15225" xr2:uid="{8EC7533F-AC1C-4BC7-A305-99682222BF96}"/>
+    <workbookView xWindow="0" yWindow="230" windowWidth="25600" windowHeight="15770" xr2:uid="{8EC7533F-AC1C-4BC7-A305-99682222BF96}"/>
   </bookViews>
   <sheets>
     <sheet name="Blad1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3" uniqueCount="3">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4" uniqueCount="4">
   <si>
     <t>Ordernummer</t>
   </si>
@@ -45,6 +45,9 @@
   </si>
   <si>
     <t>Aantal</t>
+  </si>
+  <si>
+    <t>OppervlakteBehandeling</t>
   </si>
 </sst>
 </file>
@@ -86,10 +89,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Standaard" xfId="0" builtinId="0"/>
@@ -424,24 +426,29 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EEB08457-C744-4E15-95E8-598B9FED179F}">
-  <dimension ref="A1:C1"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:D1"/>
+  <sheetFormatPr defaultColWidth="9.1796875" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="16.5703125" style="2" customWidth="1"/>
-    <col min="2" max="2" width="14.28515625" style="2" customWidth="1"/>
-    <col min="3" max="3" width="9.140625" style="2"/>
-    <col min="4" max="16384" width="9.140625" style="1"/>
+    <col min="1" max="1" width="16.54296875" customWidth="1"/>
+    <col min="2" max="2" width="14.26953125" customWidth="1"/>
+    <col min="3" max="3" width="9.1796875" customWidth="1"/>
+    <col min="4" max="4" width="23" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="9.1796875" style="1" customWidth="1"/>
+    <col min="6" max="16384" width="9.1796875" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A1" s="2" t="s">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="2" t="s">
+      <c r="B1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="2" t="s">
+      <c r="C1" t="s">
         <v>2</v>
+      </c>
+      <c r="D1" t="s">
+        <v>3</v>
       </c>
     </row>
   </sheetData>

</xml_diff>